<commit_message>
Translate project to English, Model E notebooks 01-05, plate experiments, final README
</commit_message>
<xml_diff>
--- a/data/interim/molecules_unique_updated.xlsx
+++ b/data/interim/molecules_unique_updated.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14856" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -49,7 +50,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -412,11 +413,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M185"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="21.44140625" customWidth="1" min="7" max="7"/>
-  </cols>
+  <dimension ref="A1:M195"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -8120,7 +8118,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>BlueBird</t>
+          <t>PFP</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -8130,30 +8128,50 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>(+)-3-METHYL-2-PHENYLBUTYRIC-ACID</t>
+          <t>1-Benzylpiperidine</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>3508-94-9</t>
+          <t>2905-56-8</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>4.998</v>
+        <v>2.972</v>
       </c>
       <c r="F146" t="n">
         <v>1</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>matrix ID BlueBird 1</t>
+          <t>matrix ID PFP 1</t>
+        </is>
+      </c>
+      <c r="H146" t="n">
+        <v>1</v>
+      </c>
+      <c r="I146" t="n">
+        <v>1</v>
+      </c>
+      <c r="J146" t="n">
+        <v>1</v>
+      </c>
+      <c r="K146" t="n">
+        <v>1</v>
+      </c>
+      <c r="L146" t="n">
+        <v>1</v>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>C1CCN(CC1)CC2=CC=CC=C2</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>BlueBird</t>
+          <t>PFP</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -8163,30 +8181,50 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>(-)-Dihydroquinine</t>
+          <t>4-(Trifluoromethyl)benzylamine</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>522-66-7</t>
+          <t>3300-51-4</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>3.348</v>
+        <v>3.315</v>
       </c>
       <c r="F147" t="n">
         <v>1</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>matrix ID BlueBird 1</t>
+          <t>matrix ID PFP 1</t>
+        </is>
+      </c>
+      <c r="H147" t="n">
+        <v>1</v>
+      </c>
+      <c r="I147" t="n">
+        <v>1</v>
+      </c>
+      <c r="J147" t="n">
+        <v>1</v>
+      </c>
+      <c r="K147" t="n">
+        <v>1</v>
+      </c>
+      <c r="L147" t="n">
+        <v>1</v>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>C1=CC(=CC=C1CN)C(F)(F)F</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>BlueBird</t>
+          <t>PFP</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -8196,30 +8234,50 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>(1R,2S)-1-[(3,5-Di-tert-butyl-2-hydroxybenzylidene)amino]-2-indanol</t>
+          <t>Di-tert-butylcyclopentadiene</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>275374-67-9</t>
+          <t>120937-44-2</t>
         </is>
       </c>
       <c r="E148" t="n">
-        <v>6.583</v>
+        <v>4.495</v>
       </c>
       <c r="F148" t="n">
         <v>1</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>matrix ID BlueBird 1</t>
+          <t>matrix ID PFP 1</t>
+        </is>
+      </c>
+      <c r="H148" t="n">
+        <v>1</v>
+      </c>
+      <c r="I148" t="n">
+        <v>1</v>
+      </c>
+      <c r="J148" t="n">
+        <v>1</v>
+      </c>
+      <c r="K148" t="n">
+        <v>1</v>
+      </c>
+      <c r="L148" t="n">
+        <v>1</v>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>CC(C)(C)C1C=CC(=C1)C(C)(C)C</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>BlueBird</t>
+          <t>PFP</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -8229,30 +8287,50 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>(S)-(-)-2-(Phenylcarbamoyloxy)_propionic acid</t>
+          <t>Diethyl_dibutylmalonate</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>102936-05-0</t>
+          <t>596-75-8</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>4.392</v>
+        <v>5.916</v>
       </c>
       <c r="F149" t="n">
         <v>1</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>matrix ID BlueBird 1</t>
+          <t>matrix ID PFP 1</t>
+        </is>
+      </c>
+      <c r="H149" t="n">
+        <v>1</v>
+      </c>
+      <c r="I149" t="n">
+        <v>1</v>
+      </c>
+      <c r="J149" t="n">
+        <v>1</v>
+      </c>
+      <c r="K149" t="n">
+        <v>1</v>
+      </c>
+      <c r="L149" t="n">
+        <v>1</v>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>CCCCC(CCCC)(C(=O)OCC)C(=O)OCC</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>BlueBird</t>
+          <t>PFP</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -8262,30 +8340,50 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>1,6-Dihydroxynaphthalene</t>
+          <t>Dimethyl-propargylmalonate</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>575-44-0</t>
+          <t>95124-07-5</t>
         </is>
       </c>
       <c r="E150" t="n">
-        <v>4.156</v>
+        <v>4.303</v>
       </c>
       <c r="F150" t="n">
         <v>1</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>matrix ID BlueBird 1</t>
+          <t>matrix ID PFP 1</t>
+        </is>
+      </c>
+      <c r="H150" t="n">
+        <v>1</v>
+      </c>
+      <c r="I150" t="n">
+        <v>1</v>
+      </c>
+      <c r="J150" t="n">
+        <v>1</v>
+      </c>
+      <c r="K150" t="n">
+        <v>1</v>
+      </c>
+      <c r="L150" t="n">
+        <v>1</v>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>COC(=O)C(CC#C)C(=O)OC</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>BlueBird</t>
+          <t>PolarTec</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -8295,30 +8393,50 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>1-Hydroxy-2-naphthoic-acid</t>
+          <t>1-BROMO-3-METHYLBUTANE</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>86-48-6</t>
+          <t>107-82-4</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>5.808</v>
+        <v>6.308</v>
       </c>
       <c r="F151" t="n">
         <v>1</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>matrix ID BlueBird 1</t>
+          <t>matrix ID PolarTec 1</t>
+        </is>
+      </c>
+      <c r="H151" t="n">
+        <v>1</v>
+      </c>
+      <c r="I151" t="n">
+        <v>1</v>
+      </c>
+      <c r="J151" t="n">
+        <v>1</v>
+      </c>
+      <c r="K151" t="n">
+        <v>1</v>
+      </c>
+      <c r="L151" t="n">
+        <v>1</v>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>CC(C)CCBr</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>BlueBird</t>
+          <t>PolarTec</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -8328,23 +8446,43 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>1-Methylisatin</t>
+          <t>Allyl-alpha-D-glucopyranoside</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>2058-74-4</t>
+          <t>7464-56-4</t>
         </is>
       </c>
       <c r="E152" t="n">
-        <v>4.016</v>
+        <v>1.204</v>
       </c>
       <c r="F152" t="n">
         <v>1</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>matrix ID BlueBird 1</t>
+          <t>matrix ID PolarTec 1</t>
+        </is>
+      </c>
+      <c r="H152" t="n">
+        <v>1</v>
+      </c>
+      <c r="I152" t="n">
+        <v>0</v>
+      </c>
+      <c r="J152" t="n">
+        <v>1</v>
+      </c>
+      <c r="K152" t="n">
+        <v>0</v>
+      </c>
+      <c r="L152" t="n">
+        <v>0</v>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>C=CCO[C@@H]1[C@@H]([C@H]([C@@H]([C@H](O1)CO)O)O)O</t>
         </is>
       </c>
     </row>
@@ -8361,16 +8499,16 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2',3',4',5',6'-Pentafluoroacetophenone</t>
+          <t>(+)-3-METHYL-2-PHENYLBUTYRIC-ACID</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>652-29-9</t>
+          <t>3508-94-9</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>5.21</v>
+        <v>4.998</v>
       </c>
       <c r="F153" t="n">
         <v>1</v>
@@ -8378,6 +8516,26 @@
       <c r="G153" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H153" t="n">
+        <v>1</v>
+      </c>
+      <c r="I153" t="n">
+        <v>1</v>
+      </c>
+      <c r="J153" t="n">
+        <v>1</v>
+      </c>
+      <c r="K153" t="n">
+        <v>1</v>
+      </c>
+      <c r="L153" t="n">
+        <v>1</v>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>CC(C)C(C1=CC=CC=C1)C(=O)O</t>
         </is>
       </c>
     </row>
@@ -8394,16 +8552,16 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2,2'-Iminodibenzoic acid</t>
+          <t>(-)-Dihydroquinine</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>579-92-0</t>
+          <t>522-66-7</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>4.886</v>
+        <v>3.348</v>
       </c>
       <c r="F154" t="n">
         <v>1</v>
@@ -8411,6 +8569,26 @@
       <c r="G154" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H154" t="n">
+        <v>1</v>
+      </c>
+      <c r="I154" t="n">
+        <v>0</v>
+      </c>
+      <c r="J154" t="n">
+        <v>0</v>
+      </c>
+      <c r="K154" t="n">
+        <v>1</v>
+      </c>
+      <c r="L154" t="n">
+        <v>1</v>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>CC[C@H]1CN2CC[C@H]1C[C@H]2[C@@H](C3=C4C=C(C=CC4=NC=C3)OC)O</t>
         </is>
       </c>
     </row>
@@ -8427,16 +8605,16 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2-Amino-4-chlorobenzoic acid</t>
+          <t>(1R,2S)-1-[(3,5-Di-tert-butyl-2-hydroxybenzylidene)amino]-2-indanol</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>89-77-0</t>
+          <t>275374-67-9</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>4.602</v>
+        <v>6.583</v>
       </c>
       <c r="F155" t="n">
         <v>1</v>
@@ -8444,6 +8622,26 @@
       <c r="G155" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H155" t="n">
+        <v>1</v>
+      </c>
+      <c r="I155" t="n">
+        <v>1</v>
+      </c>
+      <c r="J155" t="n">
+        <v>0</v>
+      </c>
+      <c r="K155" t="n">
+        <v>1</v>
+      </c>
+      <c r="L155" t="n">
+        <v>1</v>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>CC(C)(C)C1=CC(=C(C(=C1)C(C)(C)C)O)C=N[C@H]2[C@H](CC3=CC=CC=C23)O</t>
         </is>
       </c>
     </row>
@@ -8460,16 +8658,16 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2-Bromo-5-(trifluoromethyl)phenol</t>
+          <t>(S)-(-)-2-(Phenylcarbamoyloxy)_propionic acid</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>402-05-1</t>
+          <t>102936-05-0</t>
         </is>
       </c>
       <c r="E156" t="n">
-        <v>5.266</v>
+        <v>4.392</v>
       </c>
       <c r="F156" t="n">
         <v>1</v>
@@ -8477,6 +8675,26 @@
       <c r="G156" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H156" t="n">
+        <v>1</v>
+      </c>
+      <c r="I156" t="n">
+        <v>1</v>
+      </c>
+      <c r="J156" t="n">
+        <v>1</v>
+      </c>
+      <c r="K156" t="n">
+        <v>0</v>
+      </c>
+      <c r="L156" t="n">
+        <v>1</v>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>C[C@@H](C(=O)O)OC(=O)NC1=CC=CC=C1</t>
         </is>
       </c>
     </row>
@@ -8493,16 +8711,16 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2-Methyl-5-(trifluoromethyl)benzoic acid</t>
+          <t>1,6-Dihydroxynaphthalene</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>13055-63-5</t>
+          <t>575-44-0</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>5.069</v>
+        <v>4.156</v>
       </c>
       <c r="F157" t="n">
         <v>1</v>
@@ -8510,6 +8728,26 @@
       <c r="G157" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H157" t="n">
+        <v>1</v>
+      </c>
+      <c r="I157" t="n">
+        <v>1</v>
+      </c>
+      <c r="J157" t="n">
+        <v>1</v>
+      </c>
+      <c r="K157" t="n">
+        <v>0</v>
+      </c>
+      <c r="L157" t="n">
+        <v>0</v>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>C1=CC2=C(C=CC(=C2)O)C(=C1)O</t>
         </is>
       </c>
     </row>
@@ -8526,16 +8764,16 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>3'-(Trifluoromethyl)acetophenone</t>
+          <t>1-Hydroxy-2-naphthoic-acid</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>349-76-8</t>
+          <t>86-48-6</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>5.214</v>
+        <v>5.808</v>
       </c>
       <c r="F158" t="n">
         <v>1</v>
@@ -8543,6 +8781,26 @@
       <c r="G158" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H158" t="n">
+        <v>1</v>
+      </c>
+      <c r="I158" t="n">
+        <v>0</v>
+      </c>
+      <c r="J158" t="n">
+        <v>0</v>
+      </c>
+      <c r="K158" t="n">
+        <v>0</v>
+      </c>
+      <c r="L158" t="n">
+        <v>0</v>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>C1=CC=C2C(=C1)C=CC(=C2O)C(=O)O</t>
         </is>
       </c>
     </row>
@@ -8559,16 +8817,16 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>3,3'-Dimethylbisphenol_A</t>
+          <t>1-Methylisatin</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>79-97-0</t>
+          <t>2058-74-4</t>
         </is>
       </c>
       <c r="E159" t="n">
-        <v>5.221</v>
+        <v>4.016</v>
       </c>
       <c r="F159" t="n">
         <v>1</v>
@@ -8576,6 +8834,26 @@
       <c r="G159" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H159" t="n">
+        <v>1</v>
+      </c>
+      <c r="I159" t="n">
+        <v>1</v>
+      </c>
+      <c r="J159" t="n">
+        <v>0</v>
+      </c>
+      <c r="K159" t="n">
+        <v>1</v>
+      </c>
+      <c r="L159" t="n">
+        <v>1</v>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>CN1C2=CC=CC=C2C(=O)C1=O</t>
         </is>
       </c>
     </row>
@@ -8592,16 +8870,16 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>3,4,5-Trimethoxycinnamic acid</t>
+          <t>2',3',4',5',6'-Pentafluoroacetophenone</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>90-50-6</t>
+          <t>652-29-9</t>
         </is>
       </c>
       <c r="E160" t="n">
-        <v>4.373</v>
+        <v>5.21</v>
       </c>
       <c r="F160" t="n">
         <v>1</v>
@@ -8611,6 +8889,12 @@
           <t>matrix ID BlueBird 1</t>
         </is>
       </c>
+      <c r="H160" t="inlineStr"/>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="inlineStr"/>
+      <c r="M160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -8625,16 +8909,16 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>3,5-Dimethoxybenzyl-bromide</t>
+          <t>2,2'-Iminodibenzoic acid</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>877-88-3</t>
+          <t>579-92-0</t>
         </is>
       </c>
       <c r="E161" t="n">
-        <v>5.424</v>
+        <v>4.886</v>
       </c>
       <c r="F161" t="n">
         <v>1</v>
@@ -8642,13 +8926,33 @@
       <c r="G161" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H161" t="n">
+        <v>0</v>
+      </c>
+      <c r="I161" t="n">
+        <v>0</v>
+      </c>
+      <c r="J161" t="n">
+        <v>0</v>
+      </c>
+      <c r="K161" t="n">
+        <v>0</v>
+      </c>
+      <c r="L161" t="n">
+        <v>0</v>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>C1=CC=C(C(=C1)C(=O)O)NC2=CC=CC=C2C(=O)O</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>BlueBird</t>
+          <t>PFP</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -8658,23 +8962,43 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>3-(3-Fluorophenyl)propionic-acid</t>
+          <t>2,3-Dibromopropionic-acid</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>458-45-7</t>
+          <t>600-05-5</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>4.558</v>
+        <v>1.404</v>
       </c>
       <c r="F162" t="n">
         <v>1</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>matrix ID BlueBird 1</t>
+          <t>matrix ID PFP 1</t>
+        </is>
+      </c>
+      <c r="H162" t="n">
+        <v>1</v>
+      </c>
+      <c r="I162" t="n">
+        <v>1</v>
+      </c>
+      <c r="J162" t="n">
+        <v>1</v>
+      </c>
+      <c r="K162" t="n">
+        <v>1</v>
+      </c>
+      <c r="L162" t="n">
+        <v>1</v>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>C(C(C(=O)O)Br)Br</t>
         </is>
       </c>
     </row>
@@ -8691,16 +9015,16 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>3-Bromo-4-hydroxybenzoic-acid</t>
+          <t>2-Amino-4-chlorobenzoic acid</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>14348-41-5</t>
+          <t>89-77-0</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>4.052</v>
+        <v>4.602</v>
       </c>
       <c r="F163" t="n">
         <v>1</v>
@@ -8708,13 +9032,33 @@
       <c r="G163" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H163" t="n">
+        <v>1</v>
+      </c>
+      <c r="I163" t="n">
+        <v>0</v>
+      </c>
+      <c r="J163" t="n">
+        <v>1</v>
+      </c>
+      <c r="K163" t="n">
+        <v>0</v>
+      </c>
+      <c r="L163" t="n">
+        <v>0</v>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>C1=CC(=C(C=C1Cl)N)C(=O)O</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>BlueBird</t>
+          <t>PFP</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -8724,23 +9068,43 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>3-Hydroxyflavone</t>
+          <t>2-Bromo-4-iodopyridine</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>577-85-5</t>
+          <t>100523-96-4</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>5.478</v>
+        <v>4.824</v>
       </c>
       <c r="F164" t="n">
         <v>1</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>matrix ID BlueBird 1</t>
+          <t>matrix ID PFP 1</t>
+        </is>
+      </c>
+      <c r="H164" t="n">
+        <v>1</v>
+      </c>
+      <c r="I164" t="n">
+        <v>1</v>
+      </c>
+      <c r="J164" t="n">
+        <v>0</v>
+      </c>
+      <c r="K164" t="n">
+        <v>1</v>
+      </c>
+      <c r="L164" t="n">
+        <v>1</v>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>C1=CN=C(C=C1I)Br</t>
         </is>
       </c>
     </row>
@@ -8757,16 +9121,16 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>4'-(4-Methoxyphenyl)-2,2':6',2''-terpyridine</t>
+          <t>2-Bromo-5-(trifluoromethyl)phenol</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>13104-56-8</t>
+          <t>402-05-1</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>6.028</v>
+        <v>5.266</v>
       </c>
       <c r="F165" t="n">
         <v>1</v>
@@ -8774,6 +9138,26 @@
       <c r="G165" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H165" t="n">
+        <v>1</v>
+      </c>
+      <c r="I165" t="n">
+        <v>1</v>
+      </c>
+      <c r="J165" t="n">
+        <v>1</v>
+      </c>
+      <c r="K165" t="n">
+        <v>1</v>
+      </c>
+      <c r="L165" t="n">
+        <v>1</v>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>C1=CC(=C(C=C1C(F)(F)F)O)Br</t>
         </is>
       </c>
     </row>
@@ -8790,16 +9174,16 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>4'-Bromoacetophenone</t>
+          <t>2-Methyl-5-(trifluoromethyl)benzoic acid</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>99-90-1</t>
+          <t>13055-63-5</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>5.114</v>
+        <v>5.069</v>
       </c>
       <c r="F166" t="n">
         <v>1</v>
@@ -8807,6 +9191,26 @@
       <c r="G166" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H166" t="n">
+        <v>1</v>
+      </c>
+      <c r="I166" t="n">
+        <v>1</v>
+      </c>
+      <c r="J166" t="n">
+        <v>1</v>
+      </c>
+      <c r="K166" t="n">
+        <v>1</v>
+      </c>
+      <c r="L166" t="n">
+        <v>1</v>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>CC1=C(C=C(C=C1)C(F)(F)F)C(=O)O</t>
         </is>
       </c>
     </row>
@@ -8823,16 +9227,16 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>4-(Decyloxy)benzoic-acid</t>
+          <t>3'-(Trifluoromethyl)acetophenone</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>5519-23-3</t>
+          <t>349-76-8</t>
         </is>
       </c>
       <c r="E167" t="n">
-        <v>6.603</v>
+        <v>5.214</v>
       </c>
       <c r="F167" t="n">
         <v>1</v>
@@ -8842,6 +9246,12 @@
           <t>matrix ID BlueBird 1</t>
         </is>
       </c>
+      <c r="H167" t="inlineStr"/>
+      <c r="I167" t="inlineStr"/>
+      <c r="J167" t="inlineStr"/>
+      <c r="K167" t="inlineStr"/>
+      <c r="L167" t="inlineStr"/>
+      <c r="M167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -8856,16 +9266,16 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>4-(trifluoromethyl)benzylamine</t>
+          <t>3,3'-Dimethylbisphenol_A</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>3300-51-4</t>
+          <t>79-97-0</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>1.615</v>
+        <v>5.221</v>
       </c>
       <c r="F168" t="n">
         <v>1</v>
@@ -8873,6 +9283,26 @@
       <c r="G168" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H168" t="n">
+        <v>1</v>
+      </c>
+      <c r="I168" t="n">
+        <v>1</v>
+      </c>
+      <c r="J168" t="n">
+        <v>1</v>
+      </c>
+      <c r="K168" t="n">
+        <v>1</v>
+      </c>
+      <c r="L168" t="n">
+        <v>1</v>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>CC1=C(C=CC(=C1)C(C)(C)C2=CC(=C(C=C2)O)C)O</t>
         </is>
       </c>
     </row>
@@ -8889,16 +9319,16 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>4-Bromo-2,6-di-tert-butylphenol</t>
+          <t>3,4,5-Trimethoxycinnamic acid</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>1139-52-2</t>
+          <t>90-50-6</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>6.615</v>
+        <v>4.373</v>
       </c>
       <c r="F169" t="n">
         <v>1</v>
@@ -8906,13 +9336,33 @@
       <c r="G169" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H169" t="n">
+        <v>1</v>
+      </c>
+      <c r="I169" t="n">
+        <v>1</v>
+      </c>
+      <c r="J169" t="n">
+        <v>1</v>
+      </c>
+      <c r="K169" t="n">
+        <v>1</v>
+      </c>
+      <c r="L169" t="n">
+        <v>1</v>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>COC1=CC(=CC(=C1OC)OC)/C=C/C(=O)O</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>BlueBird</t>
+          <t>PFP</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -8922,23 +9372,43 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>4-Chloro-3-methoxybenzaldehyde</t>
+          <t>3,4-Diacetoxybenzaldehyde</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>13726-16-4</t>
+          <t>67727-64-4</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>5.012</v>
+        <v>4.513</v>
       </c>
       <c r="F170" t="n">
         <v>1</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>matrix ID BlueBird 1</t>
+          <t>matrix ID PFP 1</t>
+        </is>
+      </c>
+      <c r="H170" t="n">
+        <v>1</v>
+      </c>
+      <c r="I170" t="n">
+        <v>1</v>
+      </c>
+      <c r="J170" t="n">
+        <v>1</v>
+      </c>
+      <c r="K170" t="n">
+        <v>1</v>
+      </c>
+      <c r="L170" t="n">
+        <v>1</v>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>CC(=O)OC1=C(C=C(C=C1)C=O)OC(=O)C</t>
         </is>
       </c>
     </row>
@@ -8955,16 +9425,16 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>4-Hydroxy-4'-isopropoxydiphenylsulfone</t>
+          <t>3,5-Dimethoxybenzyl-bromide</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>95235-30-6</t>
+          <t>877-88-3</t>
         </is>
       </c>
       <c r="E171" t="n">
-        <v>5.076</v>
+        <v>5.424</v>
       </c>
       <c r="F171" t="n">
         <v>1</v>
@@ -8974,6 +9444,12 @@
           <t>matrix ID BlueBird 1</t>
         </is>
       </c>
+      <c r="H171" t="inlineStr"/>
+      <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr"/>
+      <c r="M171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -8988,16 +9464,16 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>4-Methoxybenzoyl_chloride</t>
+          <t>3-(3-Fluorophenyl)propionic-acid</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>100-07-2</t>
+          <t>458-45-7</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>4.192</v>
+        <v>4.558</v>
       </c>
       <c r="F172" t="n">
         <v>1</v>
@@ -9005,6 +9481,26 @@
       <c r="G172" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H172" t="n">
+        <v>1</v>
+      </c>
+      <c r="I172" t="n">
+        <v>1</v>
+      </c>
+      <c r="J172" t="n">
+        <v>1</v>
+      </c>
+      <c r="K172" t="n">
+        <v>1</v>
+      </c>
+      <c r="L172" t="n">
+        <v>1</v>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>C1=CC(=CC(=C1)F)CCC(=O)O</t>
         </is>
       </c>
     </row>
@@ -9021,16 +9517,16 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>5-Methoxy-2-methylindole</t>
+          <t>3-Bromo-4-hydroxybenzoic-acid</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>1076-74-0</t>
+          <t>14348-41-5</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>4.95</v>
+        <v>4.052</v>
       </c>
       <c r="F173" t="n">
         <v>1</v>
@@ -9038,6 +9534,26 @@
       <c r="G173" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H173" t="n">
+        <v>1</v>
+      </c>
+      <c r="I173" t="n">
+        <v>1</v>
+      </c>
+      <c r="J173" t="n">
+        <v>1</v>
+      </c>
+      <c r="K173" t="n">
+        <v>0</v>
+      </c>
+      <c r="L173" t="n">
+        <v>0</v>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>C1=CC(=C(C=C1C(=O)O)Br)O</t>
         </is>
       </c>
     </row>
@@ -9054,16 +9570,16 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Benzoic acid,4-amino-3-hydroxy-,methyl ester</t>
+          <t>3-Hydroxyflavone</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>63435-16-5</t>
+          <t>577-85-5</t>
         </is>
       </c>
       <c r="E174" t="n">
-        <v>3.775</v>
+        <v>5.478</v>
       </c>
       <c r="F174" t="n">
         <v>1</v>
@@ -9071,6 +9587,26 @@
       <c r="G174" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H174" t="n">
+        <v>0</v>
+      </c>
+      <c r="I174" t="n">
+        <v>0</v>
+      </c>
+      <c r="J174" t="n">
+        <v>0</v>
+      </c>
+      <c r="K174" t="n">
+        <v>1</v>
+      </c>
+      <c r="L174" t="n">
+        <v>1</v>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>C1=CC=C(C=C1)C2=C(C(=O)C3=CC=CC=C3O2)O</t>
         </is>
       </c>
     </row>
@@ -9087,16 +9623,16 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Benzyl-sulfone</t>
+          <t>4'-(4-Methoxyphenyl)-2,2':6',2''-terpyridine</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>620-32-6</t>
+          <t>13104-56-8</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>5.072</v>
+        <v>6.028</v>
       </c>
       <c r="F175" t="n">
         <v>1</v>
@@ -9104,6 +9640,26 @@
       <c r="G175" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H175" t="n">
+        <v>0</v>
+      </c>
+      <c r="I175" t="n">
+        <v>0</v>
+      </c>
+      <c r="J175" t="n">
+        <v>0</v>
+      </c>
+      <c r="K175" t="n">
+        <v>1</v>
+      </c>
+      <c r="L175" t="n">
+        <v>1</v>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>COC1=CC=C(C=C1)C2=CC(=NC(=C2)C3=CC=CC=N3)C4=CC=CC=N4</t>
         </is>
       </c>
     </row>
@@ -9120,16 +9676,16 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Biphenyl-4-sulfonyl-chloride</t>
+          <t>4'-Bromoacetophenone</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>1623-93-4</t>
+          <t>99-90-1</t>
         </is>
       </c>
       <c r="E176" t="n">
-        <v>6.006</v>
+        <v>5.114</v>
       </c>
       <c r="F176" t="n">
         <v>1</v>
@@ -9137,13 +9693,33 @@
       <c r="G176" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H176" t="n">
+        <v>1</v>
+      </c>
+      <c r="I176" t="n">
+        <v>1</v>
+      </c>
+      <c r="J176" t="n">
+        <v>1</v>
+      </c>
+      <c r="K176" t="n">
+        <v>1</v>
+      </c>
+      <c r="L176" t="n">
+        <v>1</v>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>CC(=O)C1=CC=C(C=C1)Br</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>BlueBird</t>
+          <t>PFP</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -9153,23 +9729,43 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Butyl sulfone</t>
+          <t>4-(2-Keto-1-benzimidazolinyl)piperidine</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>598-04-9</t>
+          <t>20662-53-7</t>
         </is>
       </c>
       <c r="E177" t="n">
-        <v>4.753</v>
+        <v>2.306</v>
       </c>
       <c r="F177" t="n">
         <v>1</v>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>matrix ID BlueBird 1</t>
+          <t>matrix ID PFP 1</t>
+        </is>
+      </c>
+      <c r="H177" t="n">
+        <v>1</v>
+      </c>
+      <c r="I177" t="n">
+        <v>0</v>
+      </c>
+      <c r="J177" t="n">
+        <v>0</v>
+      </c>
+      <c r="K177" t="n">
+        <v>1</v>
+      </c>
+      <c r="L177" t="n">
+        <v>1</v>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>C1CNCCC1N2C3=CC=CC=C3NC2=O</t>
         </is>
       </c>
     </row>
@@ -9186,16 +9782,16 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>D-Sphingosine</t>
+          <t>4-(Decyloxy)benzoic-acid</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>123-78-4</t>
+          <t>5519-23-3</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>4.447</v>
+        <v>6.603</v>
       </c>
       <c r="F178" t="n">
         <v>1</v>
@@ -9203,6 +9799,26 @@
       <c r="G178" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H178" t="n">
+        <v>0</v>
+      </c>
+      <c r="I178" t="n">
+        <v>0</v>
+      </c>
+      <c r="J178" t="n">
+        <v>0</v>
+      </c>
+      <c r="K178" t="n">
+        <v>0</v>
+      </c>
+      <c r="L178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>CCCCCCCCCCOC1=CC=C(C=C1)C(=O)O</t>
         </is>
       </c>
     </row>
@@ -9219,16 +9835,16 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Di-tert-Butyl-m-cresol</t>
+          <t>4-Bromo-2,6-di-tert-butylphenol</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>497-39-2</t>
+          <t>1139-52-2</t>
         </is>
       </c>
       <c r="E179" t="n">
-        <v>6.246</v>
+        <v>6.615</v>
       </c>
       <c r="F179" t="n">
         <v>1</v>
@@ -9236,6 +9852,26 @@
       <c r="G179" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H179" t="n">
+        <v>1</v>
+      </c>
+      <c r="I179" t="n">
+        <v>1</v>
+      </c>
+      <c r="J179" t="n">
+        <v>0</v>
+      </c>
+      <c r="K179" t="n">
+        <v>1</v>
+      </c>
+      <c r="L179" t="n">
+        <v>1</v>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>CC(C)(C)C1=CC(=CC(=C1O)C(C)(C)C)Br</t>
         </is>
       </c>
     </row>
@@ -9252,16 +9888,16 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Ethyl-6-chloropyridine-3-carboxylate</t>
+          <t>4-Chloro-3-methoxybenzaldehyde</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>49608-01-7</t>
+          <t>13726-16-4</t>
         </is>
       </c>
       <c r="E180" t="n">
-        <v>4.953</v>
+        <v>5.012</v>
       </c>
       <c r="F180" t="n">
         <v>1</v>
@@ -9269,6 +9905,26 @@
       <c r="G180" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H180" t="n">
+        <v>1</v>
+      </c>
+      <c r="I180" t="n">
+        <v>1</v>
+      </c>
+      <c r="J180" t="n">
+        <v>0</v>
+      </c>
+      <c r="K180" t="n">
+        <v>1</v>
+      </c>
+      <c r="L180" t="n">
+        <v>1</v>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>COC1=C(C=CC(=C1)C=O)Cl</t>
         </is>
       </c>
     </row>
@@ -9285,16 +9941,16 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>N-Z-S-phenyl-L-cysteine</t>
+          <t>4-Hydroxy-4'-isopropoxydiphenylsulfone</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>159453-24-4</t>
+          <t>95235-30-6</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>5.313</v>
+        <v>5.076</v>
       </c>
       <c r="F181" t="n">
         <v>1</v>
@@ -9302,6 +9958,26 @@
       <c r="G181" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H181" t="n">
+        <v>1</v>
+      </c>
+      <c r="I181" t="n">
+        <v>1</v>
+      </c>
+      <c r="J181" t="n">
+        <v>1</v>
+      </c>
+      <c r="K181" t="n">
+        <v>1</v>
+      </c>
+      <c r="L181" t="n">
+        <v>1</v>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>CC(C)OC1=CC=C(C=C1)S(=O)(=O)C2=CC=C(C=C2)O</t>
         </is>
       </c>
     </row>
@@ -9318,16 +9994,16 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Resorufin</t>
+          <t>4-Methoxybenzoyl_chloride</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>635-78-9</t>
+          <t>100-07-2</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>4.065</v>
+        <v>4.192</v>
       </c>
       <c r="F182" t="n">
         <v>1</v>
@@ -9337,6 +10013,12 @@
           <t>matrix ID BlueBird 1</t>
         </is>
       </c>
+      <c r="H182" t="inlineStr"/>
+      <c r="I182" t="inlineStr"/>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
+      <c r="L182" t="inlineStr"/>
+      <c r="M182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -9351,16 +10033,16 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Thiamphenicol</t>
+          <t>5-Methoxy-2-methylindole</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>15318-45-3</t>
+          <t>1076-74-0</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>3.58</v>
+        <v>4.95</v>
       </c>
       <c r="F183" t="n">
         <v>1</v>
@@ -9368,6 +10050,26 @@
       <c r="G183" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H183" t="n">
+        <v>1</v>
+      </c>
+      <c r="I183" t="n">
+        <v>1</v>
+      </c>
+      <c r="J183" t="n">
+        <v>1</v>
+      </c>
+      <c r="K183" t="n">
+        <v>1</v>
+      </c>
+      <c r="L183" t="n">
+        <v>1</v>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>CC1=CC2=C(N1)C=CC(=C2)OC</t>
         </is>
       </c>
     </row>
@@ -9384,16 +10086,16 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Tris(4-(1H-imidazol-1-yl)phenyl)amine</t>
+          <t>Benzoic acid,4-amino-3-hydroxy-,methyl ester</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>1258947-79-3</t>
+          <t>63435-16-5</t>
         </is>
       </c>
       <c r="E184" t="n">
-        <v>2.92</v>
+        <v>3.775</v>
       </c>
       <c r="F184" t="n">
         <v>1</v>
@@ -9401,6 +10103,26 @@
       <c r="G184" t="inlineStr">
         <is>
           <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H184" t="n">
+        <v>1</v>
+      </c>
+      <c r="I184" t="n">
+        <v>0</v>
+      </c>
+      <c r="J184" t="n">
+        <v>0</v>
+      </c>
+      <c r="K184" t="n">
+        <v>0</v>
+      </c>
+      <c r="L184" t="n">
+        <v>1</v>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>COC(=O)C1=CC(=C(C=C1)N)O</t>
         </is>
       </c>
     </row>
@@ -9417,23 +10139,531 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
+          <t>Benzyl-sulfone</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>620-32-6</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>5.072</v>
+      </c>
+      <c r="F185" t="n">
+        <v>1</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H185" t="n">
+        <v>0</v>
+      </c>
+      <c r="I185" t="n">
+        <v>1</v>
+      </c>
+      <c r="J185" t="n">
+        <v>0</v>
+      </c>
+      <c r="K185" t="n">
+        <v>1</v>
+      </c>
+      <c r="L185" t="n">
+        <v>1</v>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>C1=CC=C(C=C1)CS(=O)(=O)CC2=CC=CC=C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>BlueBird</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>method_1</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Biphenyl-4-sulfonyl-chloride</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>1623-93-4</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>6.006</v>
+      </c>
+      <c r="F186" t="n">
+        <v>1</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr"/>
+      <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>BlueBird</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>method_1</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Butyl sulfone</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>598-04-9</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>4.753</v>
+      </c>
+      <c r="F187" t="n">
+        <v>1</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H187" t="n">
+        <v>1</v>
+      </c>
+      <c r="I187" t="n">
+        <v>1</v>
+      </c>
+      <c r="J187" t="n">
+        <v>1</v>
+      </c>
+      <c r="K187" t="n">
+        <v>1</v>
+      </c>
+      <c r="L187" t="n">
+        <v>1</v>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>CCCCS(=O)(=O)CCCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>BlueBird</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>method_1</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>D-Sphingosine</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>123-78-4</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>4.447</v>
+      </c>
+      <c r="F188" t="n">
+        <v>1</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr"/>
+      <c r="I188" t="inlineStr"/>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="inlineStr"/>
+      <c r="L188" t="inlineStr"/>
+      <c r="M188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>BlueBird</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>method_1</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Di-tert-Butyl-m-cresol</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>497-39-2</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>6.246</v>
+      </c>
+      <c r="F189" t="n">
+        <v>1</v>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H189" t="n">
+        <v>1</v>
+      </c>
+      <c r="I189" t="n">
+        <v>1</v>
+      </c>
+      <c r="J189" t="n">
+        <v>1</v>
+      </c>
+      <c r="K189" t="n">
+        <v>1</v>
+      </c>
+      <c r="L189" t="n">
+        <v>1</v>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>CC1=CC(=C(C=C1C(C)(C)C)C(C)(C)C)O</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>BlueBird</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>method_1</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Ethyl-6-chloropyridine-3-carboxylate</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>49608-01-7</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>4.953</v>
+      </c>
+      <c r="F190" t="n">
+        <v>1</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H190" t="n">
+        <v>1</v>
+      </c>
+      <c r="I190" t="n">
+        <v>1</v>
+      </c>
+      <c r="J190" t="n">
+        <v>1</v>
+      </c>
+      <c r="K190" t="n">
+        <v>1</v>
+      </c>
+      <c r="L190" t="n">
+        <v>1</v>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>CCOC(=O)C1=CN=C(C=C1)Cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>BlueBird</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>method_1</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>N-Z-S-phenyl-L-cysteine</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>159453-24-4</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>5.313</v>
+      </c>
+      <c r="F191" t="n">
+        <v>1</v>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H191" t="n">
+        <v>1</v>
+      </c>
+      <c r="I191" t="n">
+        <v>1</v>
+      </c>
+      <c r="J191" t="n">
+        <v>1</v>
+      </c>
+      <c r="K191" t="n">
+        <v>1</v>
+      </c>
+      <c r="L191" t="n">
+        <v>1</v>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>C1=CC=C(C=C1)COC(=O)N[C@@H](CSC2=CC=CC=C2)C(=O)O</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>BlueBird</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>method_1</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Resorufin</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>635-78-9</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>4.065</v>
+      </c>
+      <c r="F192" t="n">
+        <v>1</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H192" t="n">
+        <v>0</v>
+      </c>
+      <c r="I192" t="n">
+        <v>0</v>
+      </c>
+      <c r="J192" t="n">
+        <v>0</v>
+      </c>
+      <c r="K192" t="n">
+        <v>0</v>
+      </c>
+      <c r="L192" t="n">
+        <v>0</v>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>C1=CC2=C(C=C1O)OC3=CC(=O)C=CC3=N2</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>BlueBird</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>method_1</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Thiamphenicol</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>15318-45-3</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="F193" t="n">
+        <v>1</v>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H193" t="n">
+        <v>1</v>
+      </c>
+      <c r="I193" t="n">
+        <v>1</v>
+      </c>
+      <c r="J193" t="n">
+        <v>1</v>
+      </c>
+      <c r="K193" t="n">
+        <v>0</v>
+      </c>
+      <c r="L193" t="n">
+        <v>0</v>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>CS(=O)(=O)C1=CC=C(C=C1)[C@H]([C@@H](CO)NC(=O)C(Cl)Cl)O</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>BlueBird</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>method_1</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Tris(4-(1H-imidazol-1-yl)phenyl)amine</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>1258947-79-3</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="F194" t="n">
+        <v>1</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr"/>
+      <c r="I194" t="inlineStr"/>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr"/>
+      <c r="L194" t="inlineStr"/>
+      <c r="M194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>BlueBird</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>method_1</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
           <t>Z-Pro-OH</t>
         </is>
       </c>
-      <c r="D185" t="inlineStr">
+      <c r="D195" t="inlineStr">
         <is>
           <t>1148-11-4</t>
         </is>
       </c>
-      <c r="E185" t="n">
+      <c r="E195" t="n">
         <v>4.507</v>
       </c>
-      <c r="F185" t="n">
-        <v>1</v>
-      </c>
-      <c r="G185" t="inlineStr">
-        <is>
-          <t>matrix ID BlueBird 1</t>
+      <c r="F195" t="n">
+        <v>1</v>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>matrix ID BlueBird 1</t>
+        </is>
+      </c>
+      <c r="H195" t="n">
+        <v>1</v>
+      </c>
+      <c r="I195" t="n">
+        <v>1</v>
+      </c>
+      <c r="J195" t="n">
+        <v>1</v>
+      </c>
+      <c r="K195" t="n">
+        <v>1</v>
+      </c>
+      <c r="L195" t="n">
+        <v>1</v>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>C1C[C@H](N(C1)C(=O)OCC2=CC=CC=C2)C(=O)O</t>
         </is>
       </c>
     </row>

</xml_diff>